<commit_message>
Fix: remove non-existent 100 HB FS from active rewards
100 HB FS is not in the available bonus pool. Replaced it with €60 as
active in Wheel 4, and moved it to fake-only in Wheel 5. Regenerated xlsx.

https://claude.ai/code/session_013vAmKpWhGuqyrfNbwZZDXZ
</commit_message>
<xml_diff>
--- a/bonus_wheels.xlsx
+++ b/bonus_wheels.xlsx
@@ -655,7 +655,7 @@
         <v>35</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>33.78</v>
+        <v>33.77</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>0.035</v>
@@ -1580,7 +1580,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Target: €35  |  EV: €33.78  |  Undershoot: 3.50%</t>
+          <t>Target: €35  |  EV: €33.77  |  Undershoot: 3.50%</t>
         </is>
       </c>
     </row>
@@ -1642,13 +1642,13 @@
       </c>
       <c r="D6" s="8" t="inlineStr"/>
       <c r="E6" s="7" t="n">
-        <v>0.2391</v>
+        <v>0.2626</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>5.9775</v>
+        <v>6.565</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>5.9775</v>
+        <v>6.565</v>
       </c>
     </row>
     <row r="7">
@@ -1665,13 +1665,13 @@
       </c>
       <c r="D7" s="8" t="inlineStr"/>
       <c r="E7" s="7" t="n">
-        <v>0.2136</v>
+        <v>0.2261</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>6.407999999999999</v>
+        <v>6.782999999999999</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>12.3855</v>
+        <v>13.348</v>
       </c>
     </row>
     <row r="8">
@@ -1688,13 +1688,13 @@
       </c>
       <c r="D8" s="8" t="inlineStr"/>
       <c r="E8" s="7" t="n">
-        <v>0.1863</v>
+        <v>0.1885</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>6.520499999999999</v>
+        <v>6.5975</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>18.906</v>
+        <v>19.9455</v>
       </c>
     </row>
     <row r="9">
@@ -1711,13 +1711,13 @@
       </c>
       <c r="D9" s="8" t="inlineStr"/>
       <c r="E9" s="7" t="n">
-        <v>0.1564</v>
+        <v>0.1496</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>5.865</v>
+        <v>5.61</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>24.771</v>
+        <v>25.5555</v>
       </c>
     </row>
     <row r="10">
@@ -1734,13 +1734,13 @@
       </c>
       <c r="D10" s="8" t="inlineStr"/>
       <c r="E10" s="7" t="n">
-        <v>0.1226</v>
+        <v>0.1087</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>4.904</v>
+        <v>4.348</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>29.675</v>
+        <v>29.9035</v>
       </c>
     </row>
     <row r="11">
@@ -1749,21 +1749,21 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>100 HB FS</t>
+          <t>€60</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D11" s="8" t="inlineStr"/>
       <c r="E11" s="7" t="n">
-        <v>0.08199999999999999</v>
+        <v>0.0645</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>4.1</v>
+        <v>3.87</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>33.775</v>
+        <v>33.7735</v>
       </c>
     </row>
     <row r="12">
@@ -1772,11 +1772,11 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>€60</t>
+          <t>€75</t>
         </is>
       </c>
       <c r="C12" s="12" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -1790,7 +1790,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>33.775</v>
+        <v>33.7735</v>
       </c>
     </row>
     <row r="13">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>€75</t>
+          <t>€80</t>
         </is>
       </c>
       <c r="C13" s="12" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
@@ -1817,13 +1817,13 @@
         <v>0</v>
       </c>
       <c r="G13" s="12" t="n">
-        <v>33.775</v>
+        <v>33.7735</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>Total EV: €33.78  |  Undershoot: 3.50% of €35</t>
+          <t>Total EV: €33.77  |  Undershoot: 3.50% of €35</t>
         </is>
       </c>
     </row>
@@ -1920,11 +1920,11 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>€25</t>
+          <t>100 HB FS</t>
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
@@ -1947,11 +1947,11 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>€30</t>
+          <t>€25</t>
         </is>
       </c>
       <c r="C7" s="12" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
@@ -1974,11 +1974,11 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>€35</t>
+          <t>€30</t>
         </is>
       </c>
       <c r="C8" s="12" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
@@ -2001,11 +2001,11 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>€40</t>
+          <t>€35</t>
         </is>
       </c>
       <c r="C9" s="12" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -2028,21 +2028,21 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>100 HB FS</t>
+          <t>€40</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D10" s="8" t="inlineStr"/>
       <c r="E10" s="7" t="n">
-        <v>0.3567</v>
+        <v>0.2778</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>17.835</v>
+        <v>11.112</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>17.835</v>
+        <v>11.112</v>
       </c>
     </row>
     <row r="11">
@@ -2059,13 +2059,13 @@
       </c>
       <c r="D11" s="8" t="inlineStr"/>
       <c r="E11" s="7" t="n">
-        <v>0.2905</v>
+        <v>0.2633</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>17.43</v>
+        <v>15.798</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>35.265</v>
+        <v>26.91</v>
       </c>
     </row>
     <row r="12">
@@ -2082,13 +2082,13 @@
       </c>
       <c r="D12" s="8" t="inlineStr"/>
       <c r="E12" s="7" t="n">
-        <v>0.218</v>
+        <v>0.2442</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>16.35</v>
+        <v>18.315</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>51.615</v>
+        <v>45.225</v>
       </c>
     </row>
     <row r="13">
@@ -2105,13 +2105,13 @@
       </c>
       <c r="D13" s="8" t="inlineStr"/>
       <c r="E13" s="7" t="n">
-        <v>0.1348</v>
+        <v>0.2147</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>10.784</v>
+        <v>17.176</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>62.399</v>
+        <v>62.401</v>
       </c>
     </row>
     <row r="15">

</xml_diff>